<commit_message>
auto(MT): 3h refresh 2026-05-16T04:40Z
</commit_message>
<xml_diff>
--- a/summary_2026-05-16.xlsx
+++ b/summary_2026-05-16.xlsx
@@ -46310,10 +46310,10 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="D4" s="11" t="n">
         <v>58</v>
@@ -46335,10 +46335,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C5" t="n">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="D5" t="n">
         <v>35</v>
@@ -46385,10 +46385,10 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1348</v>
+        <v>1352</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>97</v>
@@ -46414,7 +46414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I84"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -46572,7 +46572,7 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>1334583801862268</t>
+          <t>4401025156884497</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -46591,7 +46591,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Luke Said</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -46602,12 +46602,12 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Luke Said</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4401025156884497</t>
+          <t>1543180304184878</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -46626,23 +46626,23 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Luke Said</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr"/>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Luke Said</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>1543180304184878</t>
+          <t>1680974129907056</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -46677,7 +46677,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1680974129907056</t>
+          <t>1479722413058169</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -46696,7 +46696,7 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
@@ -46707,12 +46707,12 @@
       <c r="C10" s="11" t="inlineStr"/>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>1479722413058169</t>
+          <t>1426917766136513</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -46747,7 +46747,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1426917766136513</t>
+          <t>1839054247500559</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -46766,7 +46766,7 @@
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Omar Rababah</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
@@ -46777,12 +46777,12 @@
       <c r="C12" s="11" t="inlineStr"/>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Matthew Spiteri</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>1839054247500559</t>
+          <t>807330788897024</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -46801,7 +46801,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Omar Rababah</t>
+          <t>Vania Agius Tabone</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -46812,12 +46812,12 @@
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Matthew Spiteri</t>
+          <t>Vania Agius Tabone</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>807330788897024</t>
+          <t>1321288733281834</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -46836,7 +46836,7 @@
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Vania Agius Tabone</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
@@ -46847,12 +46847,12 @@
       <c r="C14" s="11" t="inlineStr"/>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Vania Agius Tabone</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>1321288733281834</t>
+          <t>1140040001637847</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -46871,23 +46871,23 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1140040001637847</t>
+          <t>1488053072699926</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -46897,7 +46897,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -46906,7 +46906,7 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Alex Borg</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
@@ -46917,12 +46917,12 @@
       <c r="C16" s="11" t="inlineStr"/>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>958905883437296</t>
+          <t>2026943771563450</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -46941,7 +46941,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -46952,12 +46952,12 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1488053072699926</t>
+          <t>1003888061994637</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -46976,7 +46976,7 @@
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
@@ -46987,12 +46987,12 @@
       <c r="C18" s="11" t="inlineStr"/>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>2026943771563450</t>
+          <t>2146428012843469</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -47011,7 +47011,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>George Vital Zammit</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -47022,12 +47022,12 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t xml:space="preserve">George Vital Zammit Kandidat PN </t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1003888061994637</t>
+          <t>864621386654273</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -47046,7 +47046,7 @@
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Luke Said</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
@@ -47057,12 +47057,12 @@
       <c r="C20" s="11" t="inlineStr"/>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Luke Said</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>2146428012843469</t>
+          <t>1527443655600364</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -47081,7 +47081,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>George Vital Zammit</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -47092,12 +47092,12 @@
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">George Vital Zammit Kandidat PN </t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>864621386654273</t>
+          <t>2423292861498917</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -47116,7 +47116,7 @@
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>Luke Said</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
@@ -47127,12 +47127,12 @@
       <c r="C22" s="11" t="inlineStr"/>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Luke Said</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>1527443655600364</t>
+          <t>1690336838632544</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -47151,7 +47151,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Frank Anthony Tabone</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -47162,12 +47162,12 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Frank Anthony Tabone</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2423292861498917</t>
+          <t>1545046643935454</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -47186,23 +47186,23 @@
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr"/>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>1690336838632544</t>
+          <t>1398617112285911</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -47221,23 +47221,23 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Frank Anthony Tabone</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Frank Anthony Tabone</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1545046643935454</t>
+          <t>1501901271598336</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -47256,7 +47256,7 @@
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
@@ -47267,12 +47267,12 @@
       <c r="C26" s="11" t="inlineStr"/>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>1398617112285911</t>
+          <t>964787089807501</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -47291,7 +47291,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -47302,12 +47302,12 @@
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1501901271598336</t>
+          <t>1862149954473065</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -47326,7 +47326,7 @@
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Carlos Zarb</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
@@ -47337,12 +47337,12 @@
       <c r="C28" s="11" t="inlineStr"/>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Carlos Zarb</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>964787089807501</t>
+          <t>939653538880289</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
@@ -47361,23 +47361,23 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1862149954473065</t>
+          <t>1463878141656116</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
@@ -47387,7 +47387,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -47396,23 +47396,23 @@
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>Carlos Zarb</t>
+          <t>Rachel Williams</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr"/>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Carlos Zarb</t>
+          <t>Williams Hymie Rubetta</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>939653538880289</t>
+          <t>1534731544699810</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
@@ -47422,7 +47422,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr"/>
@@ -47431,23 +47431,23 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1463878141656116</t>
+          <t>1531533181939436</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
@@ -47466,23 +47466,23 @@
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Joseph Grech</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr"/>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Yana Borg Debono Grech</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>1676734580000579</t>
+          <t>1246323254060158</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
@@ -47501,23 +47501,23 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Rachel Williams</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Williams Hymie Rubetta</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1534731544699810</t>
+          <t>26632426153093650</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
@@ -47536,23 +47536,23 @@
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr"/>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>1531533181939436</t>
+          <t>26732437223117722</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
@@ -47571,23 +47571,23 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Paula Mifsud Bonnici</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Maria Mifsud Bonnici</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1246323254060158</t>
+          <t>2435722906905478</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
@@ -47606,23 +47606,23 @@
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr"/>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>26632426153093650</t>
+          <t>978460398253114</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
@@ -47641,23 +47641,23 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Robert Abela</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Anthony Agius Decelis</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>26732437223117722</t>
+          <t>2064151104521171</t>
         </is>
       </c>
       <c r="F37" s="8" t="inlineStr">
@@ -47676,23 +47676,23 @@
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>Paula Mifsud Bonnici</t>
+          <t>Jesmond Bonello</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr"/>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Maria Mifsud Bonnici</t>
+          <t>Bonello Jesmond</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>2435722906905478</t>
+          <t>26918648411088542</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
@@ -47711,23 +47711,23 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>978460398253114</t>
+          <t>1504143931434748</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
@@ -47746,7 +47746,7 @@
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>Robert Abela</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
@@ -47757,12 +47757,12 @@
       <c r="C40" s="11" t="inlineStr"/>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Anthony Agius Decelis</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>2064151104521171</t>
+          <t>1518066693268355</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
@@ -47781,7 +47781,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Jesmond Bonello</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -47792,12 +47792,12 @@
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Bonello Jesmond</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>26918648411088542</t>
+          <t>1985551062067193</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
@@ -47807,7 +47807,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
@@ -47816,7 +47816,7 @@
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Tania Borg</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
@@ -47827,12 +47827,12 @@
       <c r="C42" s="11" t="inlineStr"/>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Tania Borg For District 9 &amp; 10</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>1504143931434748</t>
+          <t>974302048675707</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
@@ -47842,7 +47842,7 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr"/>
@@ -47851,7 +47851,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Tania Borg</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -47862,12 +47862,12 @@
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Tania Borg For District 9 &amp; 10</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1518066693268355</t>
+          <t>1025067929953806</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
@@ -47877,7 +47877,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H43" t="inlineStr"/>
@@ -47886,7 +47886,7 @@
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
@@ -47897,12 +47897,12 @@
       <c r="C44" s="11" t="inlineStr"/>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>1985551062067193</t>
+          <t>962084660082350</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -47921,7 +47921,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Tania Borg</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -47932,12 +47932,12 @@
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Tania Borg For District 9 &amp; 10</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>974302048675707</t>
+          <t>1430222058857743</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
@@ -47956,7 +47956,7 @@
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
         <is>
-          <t>Tania Borg</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="B46" s="11" t="inlineStr">
@@ -47967,12 +47967,12 @@
       <c r="C46" s="11" t="inlineStr"/>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Tania Borg For District 9 &amp; 10</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>1025067929953806</t>
+          <t>916777084726084</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
@@ -47991,23 +47991,23 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>962084660082350</t>
+          <t>26740161725645731</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
@@ -48026,23 +48026,23 @@
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr"/>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>1430222058857743</t>
+          <t>993445096523240</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
@@ -48052,7 +48052,7 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr"/>
@@ -48061,23 +48061,23 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>916777084726084</t>
+          <t>1006210008553971</t>
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
@@ -48087,7 +48087,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H49" t="inlineStr"/>
@@ -48096,7 +48096,7 @@
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
@@ -48107,12 +48107,12 @@
       <c r="C50" s="11" t="inlineStr"/>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>26740161725645731</t>
+          <t>2068362770561777</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
@@ -48122,7 +48122,7 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr"/>
@@ -48131,7 +48131,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -48142,12 +48142,12 @@
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>993445096523240</t>
+          <t>1645270733376689</t>
         </is>
       </c>
       <c r="F51" s="8" t="inlineStr">
@@ -48166,23 +48166,23 @@
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr"/>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>1006210008553971</t>
+          <t>996986282983288</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
@@ -48201,23 +48201,23 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Cressida Galea</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Cressida Galea - Ekonomista</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2068362770561777</t>
+          <t>4353539594976013</t>
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
@@ -48236,23 +48236,23 @@
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Cressida Galea</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr"/>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Cressida Galea - Ekonomista</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>1645270733376689</t>
+          <t>1656439582071818</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
@@ -48271,7 +48271,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Kaydem Schembri</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -48282,12 +48282,12 @@
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Kaydem Schembri</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>996986282983288</t>
+          <t>996190969523573</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
@@ -48306,23 +48306,23 @@
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
         <is>
-          <t>Cressida Galea</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr"/>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Cressida Galea - Ekonomista</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>4353539594976013</t>
+          <t>1625614571830540</t>
         </is>
       </c>
       <c r="F56" s="8" t="inlineStr">
@@ -48341,7 +48341,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Cressida Galea</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -48352,12 +48352,12 @@
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Cressida Galea - Ekonomista</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>1656439582071818</t>
+          <t>3984183268548920</t>
         </is>
       </c>
       <c r="F57" s="8" t="inlineStr">
@@ -48376,23 +48376,23 @@
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>Kaydem Schembri</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr"/>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Kaydem Schembri</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>996190969523573</t>
+          <t>3276604689166967</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
@@ -48402,7 +48402,7 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr"/>
@@ -48411,23 +48411,23 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>James Aaron Ellul</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>James Aaron Ellul</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>1625614571830540</t>
+          <t>1740543544043475</t>
         </is>
       </c>
       <c r="F59" s="8" t="inlineStr">
@@ -48437,7 +48437,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H59" t="inlineStr"/>
@@ -48446,7 +48446,7 @@
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
@@ -48457,12 +48457,12 @@
       <c r="C60" s="11" t="inlineStr"/>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
         <is>
-          <t>3984183268548920</t>
+          <t>2115618699296224</t>
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
@@ -48472,7 +48472,7 @@
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr"/>
@@ -48481,23 +48481,23 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>3276604689166967</t>
+          <t>949145677752982</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
@@ -48516,23 +48516,23 @@
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>James Aaron Ellul</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr"/>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>James Aaron Ellul</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
-          <t>1740543544043475</t>
+          <t>1470892497314849</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
@@ -48551,23 +48551,23 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2115618699296224</t>
+          <t>1997023797841290</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
@@ -48586,7 +48586,7 @@
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t>Georvin Bugeja</t>
+          <t>Lorna Borg Vassallo</t>
         </is>
       </c>
       <c r="B64" s="11" t="inlineStr">
@@ -48597,12 +48597,12 @@
       <c r="C64" s="11" t="inlineStr"/>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>Georvin Bugeja</t>
+          <t>Lorna Borġ Vassallo</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>1718685122902055</t>
+          <t>982543764707676</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
@@ -48621,23 +48621,23 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>949145677752982</t>
+          <t>35349534414693500</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
@@ -48647,7 +48647,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H65" t="inlineStr"/>
@@ -48656,23 +48656,23 @@
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr"/>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
         <is>
-          <t>1470892497314849</t>
+          <t>2489452081571575</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
@@ -48682,7 +48682,7 @@
       </c>
       <c r="G66" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H66" s="11" t="inlineStr"/>
@@ -48691,23 +48691,23 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Katya De Giovanni</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Katya De Giovanni</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>1997023797841290</t>
+          <t>26625959597085054</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
@@ -48717,7 +48717,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="H67" t="inlineStr"/>
@@ -48726,7 +48726,7 @@
     <row r="68">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borg Vassallo</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
@@ -48737,12 +48737,12 @@
       <c r="C68" s="11" t="inlineStr"/>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borġ Vassallo</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>982543764707676</t>
+          <t>1269656098669646</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
@@ -48752,7 +48752,7 @@
       </c>
       <c r="G68" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="H68" s="11" t="inlineStr"/>
@@ -48761,7 +48761,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -48772,12 +48772,12 @@
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>35349534414693500</t>
+          <t>909198525476235</t>
         </is>
       </c>
       <c r="F69" s="8" t="inlineStr">
@@ -48787,7 +48787,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="H69" t="inlineStr"/>
@@ -48812,7 +48812,7 @@
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>2489452081571575</t>
+          <t>1751227829173959</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
@@ -48822,7 +48822,7 @@
       </c>
       <c r="G70" s="11" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="H70" s="11" t="inlineStr"/>
@@ -48831,23 +48831,23 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Katya De Giovanni</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Katya De Giovanni</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>26625959597085054</t>
+          <t>1677247313280464</t>
         </is>
       </c>
       <c r="F71" s="8" t="inlineStr">
@@ -48857,7 +48857,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
@@ -48866,7 +48866,7 @@
     <row r="72">
       <c r="A72" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Nigel Vella</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
@@ -48877,12 +48877,12 @@
       <c r="C72" s="11" t="inlineStr"/>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Nigel Vella</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>1269656098669646</t>
+          <t>1478044677100859</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
@@ -48892,7 +48892,7 @@
       </c>
       <c r="G72" s="11" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="H72" s="11" t="inlineStr"/>
@@ -48901,23 +48901,23 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>909198525476235</t>
+          <t>25743656911977946</t>
         </is>
       </c>
       <c r="F73" s="8" t="inlineStr">
@@ -48927,7 +48927,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="H73" t="inlineStr"/>
@@ -48936,7 +48936,7 @@
     <row r="74">
       <c r="A74" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Lorna Borg Vassallo</t>
         </is>
       </c>
       <c r="B74" s="11" t="inlineStr">
@@ -48947,12 +48947,12 @@
       <c r="C74" s="11" t="inlineStr"/>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Lorna Borġ Vassallo</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
         <is>
-          <t>1751227829173959</t>
+          <t>942778361908557</t>
         </is>
       </c>
       <c r="F74" s="8" t="inlineStr">
@@ -48962,7 +48962,7 @@
       </c>
       <c r="G74" s="11" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="H74" s="11" t="inlineStr"/>
@@ -48971,23 +48971,23 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Lorna Borg Vassallo</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Lorna Borġ Vassallo</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>1677247313280464</t>
+          <t>984647040762034</t>
         </is>
       </c>
       <c r="F75" s="8" t="inlineStr">
@@ -48997,7 +48997,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="H75" t="inlineStr"/>
@@ -49006,7 +49006,7 @@
     <row r="76">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>Nigel Vella</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="B76" s="11" t="inlineStr">
@@ -49017,12 +49017,12 @@
       <c r="C76" s="11" t="inlineStr"/>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>Nigel Vella</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
-          <t>1478044677100859</t>
+          <t>4138793939597915</t>
         </is>
       </c>
       <c r="F76" s="8" t="inlineStr">
@@ -49032,7 +49032,7 @@
       </c>
       <c r="G76" s="11" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="H76" s="11" t="inlineStr"/>
@@ -49057,7 +49057,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>25743656911977946</t>
+          <t>992931903251467</t>
         </is>
       </c>
       <c r="F77" s="8" t="inlineStr">
@@ -49067,7 +49067,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="H77" t="inlineStr"/>
@@ -49076,7 +49076,7 @@
     <row r="78">
       <c r="A78" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borg Vassallo</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="B78" s="11" t="inlineStr">
@@ -49087,12 +49087,12 @@
       <c r="C78" s="11" t="inlineStr"/>
       <c r="D78" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borġ Vassallo</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
         <is>
-          <t>942778361908557</t>
+          <t>826788747138897</t>
         </is>
       </c>
       <c r="F78" s="8" t="inlineStr">
@@ -49102,7 +49102,7 @@
       </c>
       <c r="G78" s="11" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="H78" s="11" t="inlineStr"/>
@@ -49111,7 +49111,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Lorna Borg Vassallo</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -49122,12 +49122,12 @@
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Lorna Borġ Vassallo</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>984647040762034</t>
+          <t>866748536435658</t>
         </is>
       </c>
       <c r="F79" s="8" t="inlineStr">
@@ -49137,7 +49137,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="H79" t="inlineStr"/>
@@ -49162,7 +49162,7 @@
       </c>
       <c r="E80" s="11" t="inlineStr">
         <is>
-          <t>4138793939597915</t>
+          <t>937586149178445</t>
         </is>
       </c>
       <c r="F80" s="8" t="inlineStr">
@@ -49172,151 +49172,11 @@
       </c>
       <c r="G80" s="11" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="H80" s="11" t="inlineStr"/>
       <c r="I80" s="11" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>992931903251467</t>
-        </is>
-      </c>
-      <c r="F81" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr"/>
-      <c r="I81" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="11" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="B82" s="11" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="C82" s="11" t="inlineStr"/>
-      <c r="D82" s="11" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="E82" s="11" t="inlineStr">
-        <is>
-          <t>826788747138897</t>
-        </is>
-      </c>
-      <c r="F82" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G82" s="11" t="inlineStr">
-        <is>
-          <t>2026-04-26</t>
-        </is>
-      </c>
-      <c r="H82" s="11" t="inlineStr"/>
-      <c r="I82" s="11" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr"/>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>866748536435658</t>
-        </is>
-      </c>
-      <c r="F83" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="11" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="B84" s="11" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="C84" s="11" t="inlineStr"/>
-      <c r="D84" s="11" t="inlineStr">
-        <is>
-          <t>Lisa Cassar Shaw</t>
-        </is>
-      </c>
-      <c r="E84" s="11" t="inlineStr">
-        <is>
-          <t>937586149178445</t>
-        </is>
-      </c>
-      <c r="F84" s="8" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="G84" s="11" t="inlineStr">
-        <is>
-          <t>2026-04-23</t>
-        </is>
-      </c>
-      <c r="H84" s="11" t="inlineStr"/>
-      <c r="I84" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -49397,10 +49257,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F81" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F84" r:id="rId81"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto(MT): 3h refresh 2026-05-16T16:59Z
</commit_message>
<xml_diff>
--- a/summary_2026-05-16.xlsx
+++ b/summary_2026-05-16.xlsx
@@ -52271,10 +52271,10 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="D4" s="11" t="n">
         <v>58</v>
@@ -52296,10 +52296,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C5" t="n">
-        <v>594</v>
+        <v>588</v>
       </c>
       <c r="D5" t="n">
         <v>35</v>
@@ -52346,10 +52346,10 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1352</v>
+        <v>1344</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>97</v>
@@ -52375,7 +52375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I89"/>
+  <dimension ref="A1:I97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -52533,7 +52533,7 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>4401025156884497</t>
+          <t>1334583801862268</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -52552,7 +52552,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Luke Said</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -52563,12 +52563,12 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Luke Said</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1543180304184878</t>
+          <t>4401025156884497</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -52587,23 +52587,23 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Luke Said</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr"/>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Luke Said</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>1680974129907056</t>
+          <t>1543180304184878</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -52638,7 +52638,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1479722413058169</t>
+          <t>1680974129907056</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -52657,7 +52657,7 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
@@ -52668,12 +52668,12 @@
       <c r="C10" s="11" t="inlineStr"/>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>1426917766136513</t>
+          <t>1479722413058169</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -52708,7 +52708,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1839054247500559</t>
+          <t>1426917766136513</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -52727,7 +52727,7 @@
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>Omar Rababah</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
@@ -52738,12 +52738,12 @@
       <c r="C12" s="11" t="inlineStr"/>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Matthew Spiteri</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>807330788897024</t>
+          <t>1839054247500559</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -52762,7 +52762,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Vania Agius Tabone</t>
+          <t>Omar Rababah</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -52773,12 +52773,12 @@
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Vania Agius Tabone</t>
+          <t>Matthew Spiteri</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1321288733281834</t>
+          <t>807330788897024</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -52797,7 +52797,7 @@
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Vania Agius Tabone</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
@@ -52808,12 +52808,12 @@
       <c r="C14" s="11" t="inlineStr"/>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Vania Agius Tabone</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>1140040001637847</t>
+          <t>1321288733281834</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -52832,23 +52832,23 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>27294010593539241</t>
+          <t>1140040001637847</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -52883,7 +52883,7 @@
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>747897385011138</t>
+          <t>27294010593539241</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -52902,7 +52902,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -52913,12 +52913,12 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2380595315785369</t>
+          <t>747897385011138</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -52953,7 +52953,7 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>1683215979770872</t>
+          <t>2380595315785369</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -52988,7 +52988,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1644456073494625</t>
+          <t>1683215979770872</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -53007,7 +53007,7 @@
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>Luke Said</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
@@ -53018,12 +53018,12 @@
       <c r="C20" s="11" t="inlineStr"/>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Luke Said</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>1513928240522335</t>
+          <t>1644456073494625</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -53058,7 +53058,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>939496959088168</t>
+          <t>1513928240522335</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -53077,23 +53077,23 @@
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Luke Said</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr"/>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Luke Said</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>3871030129694577</t>
+          <t>939496959088168</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -53128,7 +53128,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>945783808284948</t>
+          <t>3871030129694577</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -53147,23 +53147,23 @@
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr"/>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>1488053072699926</t>
+          <t>945783808284948</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -53173,7 +53173,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr"/>
@@ -53182,7 +53182,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Alex Borg</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -53193,12 +53193,12 @@
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026943771563450</t>
+          <t>958905883437296</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -53217,7 +53217,7 @@
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
@@ -53228,12 +53228,12 @@
       <c r="C26" s="11" t="inlineStr"/>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>1003888061994637</t>
+          <t>1488053072699926</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -53252,7 +53252,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -53263,12 +53263,12 @@
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2146428012843469</t>
+          <t>2026943771563450</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -53287,7 +53287,7 @@
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>George Vital Zammit</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
@@ -53298,12 +53298,12 @@
       <c r="C28" s="11" t="inlineStr"/>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">George Vital Zammit Kandidat PN </t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>864621386654273</t>
+          <t>1003888061994637</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
@@ -53322,7 +53322,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Luke Said</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -53333,12 +53333,12 @@
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Luke Said</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1527443655600364</t>
+          <t>2146428012843469</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
@@ -53357,7 +53357,7 @@
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>George Vital Zammit</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
@@ -53368,12 +53368,12 @@
       <c r="C30" s="11" t="inlineStr"/>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t xml:space="preserve">George Vital Zammit Kandidat PN </t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>2423292861498917</t>
+          <t>864621386654273</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
@@ -53392,7 +53392,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Luke Said</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -53403,12 +53403,12 @@
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Luke Said</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1690336838632544</t>
+          <t>1527443655600364</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
@@ -53427,7 +53427,7 @@
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Frank Anthony Tabone</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
@@ -53438,12 +53438,12 @@
       <c r="C32" s="11" t="inlineStr"/>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Frank Anthony Tabone</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>1545046643935454</t>
+          <t>2423292861498917</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
@@ -53462,23 +53462,23 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1398617112285911</t>
+          <t>1690336838632544</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
@@ -53497,23 +53497,23 @@
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Frank Anthony Tabone</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr"/>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Frank Anthony Tabone</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>1501901271598336</t>
+          <t>1545046643935454</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
@@ -53532,7 +53532,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -53543,12 +53543,12 @@
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>964787089807501</t>
+          <t>1398617112285911</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
@@ -53567,7 +53567,7 @@
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
@@ -53578,12 +53578,12 @@
       <c r="C36" s="11" t="inlineStr"/>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Olaf McKay</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>1862149954473065</t>
+          <t>1501901271598336</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
@@ -53602,7 +53602,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Carlos Zarb</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -53613,12 +53613,12 @@
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Carlos Zarb</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>939653538880289</t>
+          <t>964787089807501</t>
         </is>
       </c>
       <c r="F37" s="8" t="inlineStr">
@@ -53637,23 +53637,23 @@
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr"/>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Olaf McKay</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>1463878141656116</t>
+          <t>1862149954473065</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
@@ -53663,7 +53663,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr"/>
@@ -53672,23 +53672,23 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Rachel Williams</t>
+          <t>Carlos Zarb</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Williams Hymie Rubetta</t>
+          <t>Carlos Zarb</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1534731544699810</t>
+          <t>939653538880289</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
@@ -53698,7 +53698,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
@@ -53707,23 +53707,23 @@
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr"/>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>1531533181939436</t>
+          <t>1463878141656116</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
@@ -53742,23 +53742,23 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Joseph Grech</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Yana Borg Debono Grech</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1246323254060158</t>
+          <t>1676734580000579</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
@@ -53777,23 +53777,23 @@
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Rachel Williams</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr"/>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Williams Hymie Rubetta</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>26632426153093650</t>
+          <t>1534731544699810</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
@@ -53812,7 +53812,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -53823,12 +53823,12 @@
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>26732437223117722</t>
+          <t>1341328164530761</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
@@ -53847,23 +53847,23 @@
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>Paula Mifsud Bonnici</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr"/>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Maria Mifsud Bonnici</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>2435722906905478</t>
+          <t>1531533181939436</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -53882,23 +53882,23 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>978460398253114</t>
+          <t>1246323254060158</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
@@ -53917,7 +53917,7 @@
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
         <is>
-          <t>Robert Abela</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="B46" s="11" t="inlineStr">
@@ -53928,12 +53928,12 @@
       <c r="C46" s="11" t="inlineStr"/>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Anthony Agius Decelis</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>2064151104521171</t>
+          <t>26632426153093650</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
@@ -53952,23 +53952,23 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Jesmond Bonello</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Bonello Jesmond</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>26918648411088542</t>
+          <t>26732437223117722</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
@@ -53987,23 +53987,23 @@
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Paula Mifsud Bonnici</t>
         </is>
       </c>
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr"/>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Maria Mifsud Bonnici</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>1504143931434748</t>
+          <t>2435722906905478</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
@@ -54022,23 +54022,23 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>1518066693268355</t>
+          <t>858503737301907</t>
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
@@ -54057,23 +54057,23 @@
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr"/>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>1985551062067193</t>
+          <t>978460398253114</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
@@ -54083,7 +54083,7 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr"/>
@@ -54092,7 +54092,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Tania Borg</t>
+          <t>Robert Abela</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -54103,12 +54103,12 @@
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Tania Borg For District 9 &amp; 10</t>
+          <t>Anthony Agius Decelis</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>974302048675707</t>
+          <t>2064151104521171</t>
         </is>
       </c>
       <c r="F51" s="8" t="inlineStr">
@@ -54118,7 +54118,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
@@ -54127,7 +54127,7 @@
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t>Tania Borg</t>
+          <t>Yana Borg Debono Grech</t>
         </is>
       </c>
       <c r="B52" s="11" t="inlineStr">
@@ -54138,12 +54138,12 @@
       <c r="C52" s="11" t="inlineStr"/>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Tania Borg For District 9 &amp; 10</t>
+          <t>Yana Borg Debono Grech</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>1025067929953806</t>
+          <t>1462425145622327</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
@@ -54153,7 +54153,7 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr"/>
@@ -54162,7 +54162,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Jesmond Bonello</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -54173,12 +54173,12 @@
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Bonello Jesmond</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>962084660082350</t>
+          <t>26918648411088542</t>
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
@@ -54188,7 +54188,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H53" t="inlineStr"/>
@@ -54197,7 +54197,7 @@
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
@@ -54208,12 +54208,12 @@
       <c r="C54" s="11" t="inlineStr"/>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Alex Muscat</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>1430222058857743</t>
+          <t>1504143931434748</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
@@ -54223,7 +54223,7 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr"/>
@@ -54232,7 +54232,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -54243,12 +54243,12 @@
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>916777084726084</t>
+          <t>1518066693268355</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
@@ -54258,7 +54258,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="H55" t="inlineStr"/>
@@ -54267,23 +54267,23 @@
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr"/>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Leone Sciberras</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>26740161725645731</t>
+          <t>1985551062067193</t>
         </is>
       </c>
       <c r="F56" s="8" t="inlineStr">
@@ -54302,23 +54302,23 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Tania Borg</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>Tania Borg For District 9 &amp; 10</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>993445096523240</t>
+          <t>974302048675707</t>
         </is>
       </c>
       <c r="F57" s="8" t="inlineStr">
@@ -54328,7 +54328,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H57" t="inlineStr"/>
@@ -54337,23 +54337,23 @@
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Tania Borg</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr"/>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Julian Borg</t>
+          <t>Tania Borg For District 9 &amp; 10</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>1006210008553971</t>
+          <t>1025067929953806</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
@@ -54363,7 +54363,7 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr"/>
@@ -54372,23 +54372,23 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Beppe Galea</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2068362770561777</t>
+          <t>962084660082350</t>
         </is>
       </c>
       <c r="F59" s="8" t="inlineStr">
@@ -54398,7 +54398,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H59" t="inlineStr"/>
@@ -54407,23 +54407,23 @@
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr"/>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Graziella Galea</t>
+          <t>Alex Muscat</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
         <is>
-          <t>1645270733376689</t>
+          <t>1430222058857743</t>
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
@@ -54433,7 +54433,7 @@
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr"/>
@@ -54442,7 +54442,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -54453,12 +54453,12 @@
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>996986282983288</t>
+          <t>916777084726084</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
@@ -54468,7 +54468,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
@@ -54477,23 +54477,23 @@
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>Cressida Galea</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr"/>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Cressida Galea - Ekonomista</t>
+          <t>Leone Sciberras</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
-          <t>4353539594976013</t>
+          <t>26740161725645731</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
@@ -54503,7 +54503,7 @@
       </c>
       <c r="G62" s="11" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr"/>
@@ -54512,23 +54512,23 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Cressida Galea</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Cressida Galea - Ekonomista</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>1656439582071818</t>
+          <t>993445096523240</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
@@ -54547,23 +54547,23 @@
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t>Kaydem Schembri</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="B64" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr"/>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>Kaydem Schembri</t>
+          <t>Julian Borg</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>996190969523573</t>
+          <t>1006210008553971</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
@@ -54582,23 +54582,23 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Beppe Galea</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>1625614571830540</t>
+          <t>2068362770561777</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
@@ -54617,23 +54617,23 @@
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr"/>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Graziella Galea</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
         <is>
-          <t>3984183268548920</t>
+          <t>1645270733376689</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
@@ -54652,23 +54652,23 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Duncan Borg Myatt</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>3276604689166967</t>
+          <t>996986282983288</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
@@ -54678,7 +54678,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H67" t="inlineStr"/>
@@ -54687,23 +54687,23 @@
     <row r="68">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>James Aaron Ellul</t>
+          <t>Cressida Galea</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C68" s="11" t="inlineStr"/>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>James Aaron Ellul</t>
+          <t>Cressida Galea - Ekonomista</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>1740543544043475</t>
+          <t>4353539594976013</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
@@ -54713,7 +54713,7 @@
       </c>
       <c r="G68" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H68" s="11" t="inlineStr"/>
@@ -54722,7 +54722,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Cressida Galea</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -54733,12 +54733,12 @@
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Ray Abela</t>
+          <t>Cressida Galea - Ekonomista</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2115618699296224</t>
+          <t>1656439582071818</t>
         </is>
       </c>
       <c r="F69" s="8" t="inlineStr">
@@ -54748,7 +54748,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H69" t="inlineStr"/>
@@ -54757,7 +54757,7 @@
     <row r="70">
       <c r="A70" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Kaydem Schembri</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
@@ -54768,12 +54768,12 @@
       <c r="C70" s="11" t="inlineStr"/>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>Edward Cassar Delia</t>
+          <t>Kaydem Schembri</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>949145677752982</t>
+          <t>996190969523573</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
@@ -54783,7 +54783,7 @@
       </c>
       <c r="G70" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H70" s="11" t="inlineStr"/>
@@ -54808,7 +54808,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>1470892497314849</t>
+          <t>1625614571830540</t>
         </is>
       </c>
       <c r="F71" s="8" t="inlineStr">
@@ -54818,7 +54818,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
@@ -54827,23 +54827,23 @@
     <row r="72">
       <c r="A72" s="11" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C72" s="11" t="inlineStr"/>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>Matthew Agius</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>1997023797841290</t>
+          <t>3984183268548920</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
@@ -54853,7 +54853,7 @@
       </c>
       <c r="G72" s="11" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H72" s="11" t="inlineStr"/>
@@ -54862,23 +54862,23 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Lorna Borg Vassallo</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Lorna Borġ Vassallo</t>
+          <t>Duncan Borg Myatt</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>982543764707676</t>
+          <t>3276604689166967</t>
         </is>
       </c>
       <c r="F73" s="8" t="inlineStr">
@@ -54897,7 +54897,7 @@
     <row r="74">
       <c r="A74" s="11" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>James Aaron Ellul</t>
         </is>
       </c>
       <c r="B74" s="11" t="inlineStr">
@@ -54908,12 +54908,12 @@
       <c r="C74" s="11" t="inlineStr"/>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>John Baptist Camilleri</t>
+          <t>James Aaron Ellul</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
         <is>
-          <t>35349534414693500</t>
+          <t>1740543544043475</t>
         </is>
       </c>
       <c r="F74" s="8" t="inlineStr">
@@ -54923,7 +54923,7 @@
       </c>
       <c r="G74" s="11" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H74" s="11" t="inlineStr"/>
@@ -54932,23 +54932,23 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>George Muscat</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>George Muscat</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>2489452081571575</t>
+          <t>1509198534334763</t>
         </is>
       </c>
       <c r="F75" s="8" t="inlineStr">
@@ -54958,7 +54958,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H75" t="inlineStr"/>
@@ -54967,7 +54967,7 @@
     <row r="76">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>Katya De Giovanni</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="B76" s="11" t="inlineStr">
@@ -54978,12 +54978,12 @@
       <c r="C76" s="11" t="inlineStr"/>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>Katya De Giovanni</t>
+          <t>Ray Abela</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
-          <t>26625959597085054</t>
+          <t>2115618699296224</t>
         </is>
       </c>
       <c r="F76" s="8" t="inlineStr">
@@ -54993,7 +54993,7 @@
       </c>
       <c r="G76" s="11" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H76" s="11" t="inlineStr"/>
@@ -55002,7 +55002,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Georvin Bugeja</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -55013,12 +55013,12 @@
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Georvin Bugeja</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>1269656098669646</t>
+          <t>1718685122902055</t>
         </is>
       </c>
       <c r="F77" s="8" t="inlineStr">
@@ -55028,7 +55028,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H77" t="inlineStr"/>
@@ -55037,23 +55037,23 @@
     <row r="78">
       <c r="A78" s="11" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="B78" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C78" s="11" t="inlineStr"/>
       <c r="D78" s="11" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Edward Cassar Delia</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
         <is>
-          <t>909198525476235</t>
+          <t>949145677752982</t>
         </is>
       </c>
       <c r="F78" s="8" t="inlineStr">
@@ -55063,7 +55063,7 @@
       </c>
       <c r="G78" s="11" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H78" s="11" t="inlineStr"/>
@@ -55072,23 +55072,23 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>1751227829173959</t>
+          <t>1470892497314849</t>
         </is>
       </c>
       <c r="F79" s="8" t="inlineStr">
@@ -55098,7 +55098,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H79" t="inlineStr"/>
@@ -55107,23 +55107,23 @@
     <row r="80">
       <c r="A80" s="11" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="B80" s="11" t="inlineStr">
         <is>
-          <t>PN</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C80" s="11" t="inlineStr"/>
       <c r="D80" s="11" t="inlineStr">
         <is>
-          <t>Michael Piccinino</t>
+          <t>Matthew Agius</t>
         </is>
       </c>
       <c r="E80" s="11" t="inlineStr">
         <is>
-          <t>1677247313280464</t>
+          <t>1997023797841290</t>
         </is>
       </c>
       <c r="F80" s="8" t="inlineStr">
@@ -55133,7 +55133,7 @@
       </c>
       <c r="G80" s="11" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H80" s="11" t="inlineStr"/>
@@ -55142,7 +55142,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Nigel Vella</t>
+          <t>Lorna Borg Vassallo</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -55153,12 +55153,12 @@
       <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Nigel Vella</t>
+          <t>Lorna Borġ Vassallo</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>1478044677100859</t>
+          <t>982543764707676</t>
         </is>
       </c>
       <c r="F81" s="8" t="inlineStr">
@@ -55168,7 +55168,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H81" t="inlineStr"/>
@@ -55177,23 +55177,23 @@
     <row r="82">
       <c r="A82" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C82" s="11" t="inlineStr"/>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>John Baptist Camilleri</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
         <is>
-          <t>25743656911977946</t>
+          <t>35349534414693500</t>
         </is>
       </c>
       <c r="F82" s="8" t="inlineStr">
@@ -55203,7 +55203,7 @@
       </c>
       <c r="G82" s="11" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H82" s="11" t="inlineStr"/>
@@ -55212,7 +55212,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Lorna Borg Vassallo</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -55223,12 +55223,12 @@
       <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Lorna Borġ Vassallo</t>
+          <t>Lisa Cassar Shaw</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>942778361908557</t>
+          <t>2489452081571575</t>
         </is>
       </c>
       <c r="F83" s="8" t="inlineStr">
@@ -55238,7 +55238,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H83" t="inlineStr"/>
@@ -55247,7 +55247,7 @@
     <row r="84">
       <c r="A84" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borg Vassallo</t>
+          <t>Katya De Giovanni</t>
         </is>
       </c>
       <c r="B84" s="11" t="inlineStr">
@@ -55258,12 +55258,12 @@
       <c r="C84" s="11" t="inlineStr"/>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>Lorna Borġ Vassallo</t>
+          <t>Katya De Giovanni</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
         <is>
-          <t>984647040762034</t>
+          <t>26625959597085054</t>
         </is>
       </c>
       <c r="F84" s="8" t="inlineStr">
@@ -55273,7 +55273,7 @@
       </c>
       <c r="G84" s="11" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="H84" s="11" t="inlineStr"/>
@@ -55298,7 +55298,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>4138793939597915</t>
+          <t>1269656098669646</t>
         </is>
       </c>
       <c r="F85" s="8" t="inlineStr">
@@ -55308,7 +55308,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="H85" t="inlineStr"/>
@@ -55317,23 +55317,23 @@
     <row r="86">
       <c r="A86" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B86" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C86" s="11" t="inlineStr"/>
       <c r="D86" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E86" s="11" t="inlineStr">
         <is>
-          <t>992931903251467</t>
+          <t>909198525476235</t>
         </is>
       </c>
       <c r="F86" s="8" t="inlineStr">
@@ -55343,7 +55343,7 @@
       </c>
       <c r="G86" s="11" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="H86" s="11" t="inlineStr"/>
@@ -55368,7 +55368,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>826788747138897</t>
+          <t>1751227829173959</t>
         </is>
       </c>
       <c r="F87" s="8" t="inlineStr">
@@ -55378,7 +55378,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="H87" t="inlineStr"/>
@@ -55387,23 +55387,23 @@
     <row r="88">
       <c r="A88" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="B88" s="11" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>PN</t>
         </is>
       </c>
       <c r="C88" s="11" t="inlineStr"/>
       <c r="D88" s="11" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Michael Piccinino</t>
         </is>
       </c>
       <c r="E88" s="11" t="inlineStr">
         <is>
-          <t>866748536435658</t>
+          <t>1677247313280464</t>
         </is>
       </c>
       <c r="F88" s="8" t="inlineStr">
@@ -55413,7 +55413,7 @@
       </c>
       <c r="G88" s="11" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="H88" s="11" t="inlineStr"/>
@@ -55422,7 +55422,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Nigel Vella</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -55433,12 +55433,12 @@
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Lisa Cassar Shaw</t>
+          <t>Nigel Vella</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>937586149178445</t>
+          <t>1478044677100859</t>
         </is>
       </c>
       <c r="F89" s="8" t="inlineStr">
@@ -55448,11 +55448,291 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="11" t="inlineStr">
+        <is>
+          <t>Lisa Cassar Shaw</t>
+        </is>
+      </c>
+      <c r="B90" s="11" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C90" s="11" t="inlineStr"/>
+      <c r="D90" s="11" t="inlineStr">
+        <is>
+          <t>Lisa Cassar Shaw</t>
+        </is>
+      </c>
+      <c r="E90" s="11" t="inlineStr">
+        <is>
+          <t>25743656911977946</t>
+        </is>
+      </c>
+      <c r="F90" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G90" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="H90" s="11" t="inlineStr"/>
+      <c r="I90" s="11" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Lorna Borg Vassallo</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Lorna Borġ Vassallo</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>942778361908557</t>
+        </is>
+      </c>
+      <c r="F91" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="11" t="inlineStr">
+        <is>
+          <t>Lorna Borg Vassallo</t>
+        </is>
+      </c>
+      <c r="B92" s="11" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C92" s="11" t="inlineStr"/>
+      <c r="D92" s="11" t="inlineStr">
+        <is>
+          <t>Lorna Borġ Vassallo</t>
+        </is>
+      </c>
+      <c r="E92" s="11" t="inlineStr">
+        <is>
+          <t>984647040762034</t>
+        </is>
+      </c>
+      <c r="F92" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G92" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="H92" s="11" t="inlineStr"/>
+      <c r="I92" s="11" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Lisa Cassar Shaw</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Lisa Cassar Shaw</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>4138793939597915</t>
+        </is>
+      </c>
+      <c r="F93" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="11" t="inlineStr">
+        <is>
+          <t>Lisa Cassar Shaw</t>
+        </is>
+      </c>
+      <c r="B94" s="11" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C94" s="11" t="inlineStr"/>
+      <c r="D94" s="11" t="inlineStr">
+        <is>
+          <t>Lisa Cassar Shaw</t>
+        </is>
+      </c>
+      <c r="E94" s="11" t="inlineStr">
+        <is>
+          <t>992931903251467</t>
+        </is>
+      </c>
+      <c r="F94" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G94" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="H94" s="11" t="inlineStr"/>
+      <c r="I94" s="11" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Lisa Cassar Shaw</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Lisa Cassar Shaw</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>826788747138897</t>
+        </is>
+      </c>
+      <c r="F95" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="11" t="inlineStr">
+        <is>
+          <t>Lisa Cassar Shaw</t>
+        </is>
+      </c>
+      <c r="B96" s="11" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C96" s="11" t="inlineStr"/>
+      <c r="D96" s="11" t="inlineStr">
+        <is>
+          <t>Lisa Cassar Shaw</t>
+        </is>
+      </c>
+      <c r="E96" s="11" t="inlineStr">
+        <is>
+          <t>866748536435658</t>
+        </is>
+      </c>
+      <c r="F96" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G96" s="11" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="H96" s="11" t="inlineStr"/>
+      <c r="I96" s="11" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Lisa Cassar Shaw</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Lisa Cassar Shaw</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>937586149178445</t>
+        </is>
+      </c>
+      <c r="F97" s="8" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -55542,6 +55822,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F87" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F88" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F89" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F90" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F91" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F92" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F93" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F94" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F95" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F96" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F97" r:id="rId94"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>